<commit_message>
feat(automatizaciones): actualizacion de cuentas de cobro, nutricion y sincronizacion de entregas RAM
</commit_message>
<xml_diff>
--- a/GENERAL_BOTS.xlsx
+++ b/GENERAL_BOTS.xlsx
@@ -1,32 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\jobautomatico\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E71304-CDD6-4DE7-8615-9841AB44F524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2565" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5580" yWindow="2565" windowWidth="21600" windowHeight="11295"/>
   </bookViews>
   <sheets>
-    <sheet name="Asociaciones" sheetId="1" r:id="rId1"/>
-    <sheet name="Jardines" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Asociaciones" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Jardines" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="253">
   <si>
     <t>Nombre Corto</t>
   </si>
@@ -692,18 +681,6 @@
   </si>
   <si>
     <t>52884517</t>
-  </si>
-  <si>
-    <t>110011120653</t>
-  </si>
-  <si>
-    <t>EL PAIS DE LAS MARAVILLAS</t>
-  </si>
-  <si>
-    <t>FANNY DEL CARMEN LUNA</t>
-  </si>
-  <si>
-    <t>20947696</t>
   </si>
   <si>
     <t>110011120642</t>
@@ -802,17 +779,24 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0;[Red]0"/>
+    <numFmt numFmtId="164" formatCode="0;[Red]0"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -836,14 +820,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1176,14 +1160,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1206,7 +1190,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1229,7 +1213,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1252,7 +1236,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1275,7 +1259,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1298,7 +1282,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1321,7 +1305,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1344,7 +1328,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1369,19 +1353,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:G5 A7:G8 A6:C6 E6:G6" numberStoredAsText="1"/>
-  </ignoredErrors>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E60"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E59"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>36</v>
       </c>
@@ -1398,7 +1379,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1415,7 +1396,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -1432,7 +1413,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -1449,7 +1430,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -1466,7 +1447,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -1483,7 +1464,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -1500,7 +1481,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -1517,7 +1498,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>59</v>
       </c>
@@ -1534,7 +1515,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>63</v>
       </c>
@@ -1551,7 +1532,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>67</v>
       </c>
@@ -1568,7 +1549,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>70</v>
       </c>
@@ -1585,7 +1566,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>74</v>
       </c>
@@ -1602,7 +1583,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>78</v>
       </c>
@@ -1619,7 +1600,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>82</v>
       </c>
@@ -1636,7 +1617,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>86</v>
       </c>
@@ -1653,7 +1634,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>90</v>
       </c>
@@ -1670,7 +1651,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>94</v>
       </c>
@@ -1687,7 +1668,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -1704,7 +1685,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>102</v>
       </c>
@@ -1721,7 +1702,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>106</v>
       </c>
@@ -1738,7 +1719,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>110</v>
       </c>
@@ -1755,7 +1736,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>114</v>
       </c>
@@ -1772,7 +1753,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>118</v>
       </c>
@@ -1789,7 +1770,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -1806,7 +1787,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>126</v>
       </c>
@@ -1823,7 +1804,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="27" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>130</v>
       </c>
@@ -1840,7 +1821,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>134</v>
       </c>
@@ -1857,7 +1838,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>138</v>
       </c>
@@ -1874,7 +1855,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>142</v>
       </c>
@@ -1891,7 +1872,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>146</v>
       </c>
@@ -1908,7 +1889,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>150</v>
       </c>
@@ -1925,7 +1906,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>154</v>
       </c>
@@ -1942,7 +1923,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>158</v>
       </c>
@@ -1959,7 +1940,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>162</v>
       </c>
@@ -1976,7 +1957,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>166</v>
       </c>
@@ -1993,7 +1974,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>170</v>
       </c>
@@ -2010,7 +1991,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>174</v>
       </c>
@@ -2027,7 +2008,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="39" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>178</v>
       </c>
@@ -2044,7 +2025,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>182</v>
       </c>
@@ -2061,7 +2042,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>182</v>
       </c>
@@ -2078,7 +2059,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>188</v>
       </c>
@@ -2095,7 +2076,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>192</v>
       </c>
@@ -2112,7 +2093,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>196</v>
       </c>
@@ -2129,7 +2110,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>196</v>
       </c>
@@ -2146,7 +2127,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>196</v>
       </c>
@@ -2163,7 +2144,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>204</v>
       </c>
@@ -2180,7 +2161,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>204</v>
       </c>
@@ -2197,7 +2178,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>210</v>
       </c>
@@ -2214,7 +2195,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>214</v>
       </c>
@@ -2231,7 +2212,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>218</v>
       </c>
@@ -2248,7 +2229,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>222</v>
       </c>
@@ -2265,7 +2246,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>226</v>
       </c>
@@ -2282,7 +2263,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>230</v>
       </c>
@@ -2293,30 +2274,30 @@
         <v>20</v>
       </c>
       <c r="D54" t="s">
+        <v>22</v>
+      </c>
+      <c r="E54" t="s">
         <v>232</v>
       </c>
-      <c r="E54" t="s">
+    </row>
+    <row r="55" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
         <v>234</v>
-      </c>
-      <c r="B55" t="s">
-        <v>235</v>
       </c>
       <c r="C55" t="s">
         <v>20</v>
       </c>
       <c r="D55" t="s">
-        <v>22</v>
+        <v>235</v>
       </c>
       <c r="E55" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>237</v>
       </c>
@@ -2333,7 +2314,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>241</v>
       </c>
@@ -2350,7 +2331,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>245</v>
       </c>
@@ -2367,7 +2348,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" ht="15.75" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>249</v>
       </c>
@@ -2384,27 +2365,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>253</v>
-      </c>
-      <c r="B60" t="s">
-        <v>254</v>
-      </c>
-      <c r="C60" t="s">
-        <v>20</v>
-      </c>
-      <c r="D60" t="s">
-        <v>255</v>
-      </c>
-      <c r="E60" t="s">
-        <v>256</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E60" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>